<commit_message>
Simply Goo's effect. Change Dart Trap's rank from 2 to 1 and adjusted the statement of its effect. Change Kamikaze Bot's rank from 2 to 1.
</commit_message>
<xml_diff>
--- a/sheet/MonsterCardData.xlsx
+++ b/sheet/MonsterCardData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{426E3936-0023-4598-A845-7CF738C46E3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64692346-BE1C-41D0-80D8-DB9EAC5B53FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4290" yWindow="3480" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -717,10 +717,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>回合结束时：如果同房间同侧没有其他怪物牌，则将主牌堆第1张怪物牌加入本牌所在房间同侧；否则移动1格。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Turret</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -734,10 +730,6 @@
   </si>
   <si>
     <t>死亡时：翻开主牌堆的“史莱姆牌”直到合计点数不小于本牌点数，然后选其中1张牌加入本牌所在房间同侧，其余的牌加入手牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>回合结束时：如果本牌点数为1，则本牌点数加1。否则本牌点数减1，然后将主牌堆第1张同名牌加入与本牌相邻的房间同侧。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -765,12 +757,21 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>回合结束时：移动1格，然后本牌点数减1。&lt;br&gt;
-本牌因点数为0而被消灭时：使同房间内所有其他牌点数减1，然后玩家受到1伤害。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>回合结束时：如果本牌所在房间没有其他牌，将本牌移动1格。否则选同房间1张其他牌，使其点数减1。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合结束时：移动1格。&lt;br&gt;
+移动时：点数减1。&lt;br&gt;
+点数为0而被消灭时：使同房间内所有其他牌点数减1，然后玩家受到1伤害。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合结束时：如果同房间同侧没有其他怪物牌，则将主牌堆第1张怪物牌加入本牌所在房间同侧，然后移动1格。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合结束时：将主牌堆第1张同名牌加入与本牌相邻的房间同侧。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1187,7 +1188,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>7</v>
@@ -1221,7 +1222,7 @@
       </c>
       <c r="H4" s="3"/>
     </row>
-    <row r="5" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>123</v>
       </c>
@@ -1229,13 +1230,13 @@
         <v>122</v>
       </c>
       <c r="C5" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" s="2">
         <v>4</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>141</v>
@@ -1259,7 +1260,7 @@
         <v>4</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>164</v>
@@ -1283,10 +1284,10 @@
         <v>4</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="3"/>
@@ -1425,7 +1426,7 @@
         <v>4</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>140</v>
@@ -1449,7 +1450,7 @@
         <v>4</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>17</v>
@@ -1461,7 +1462,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>124</v>
       </c>
@@ -1475,7 +1476,7 @@
         <v>4</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>134</v>
@@ -1499,7 +1500,7 @@
         <v>4</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>135</v>
@@ -1511,7 +1512,7 @@
     </row>
     <row r="17" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B17" t="s">
         <v>15</v>
@@ -1523,7 +1524,7 @@
         <v>4</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>136</v>
@@ -1924,7 +1925,7 @@
         <v>4</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>104</v>
@@ -2143,7 +2144,7 @@
         <v>4</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>80</v>

</xml_diff>

<commit_message>
Changed rank and effect of tower slime. Change effect of fused slime. Change effect of sentinel drone. Change effect of carrier drone. Change effect of miner bot.
</commit_message>
<xml_diff>
--- a/sheet/MonsterCardData.xlsx
+++ b/sheet/MonsterCardData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64692346-BE1C-41D0-80D8-DB9EAC5B53FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E6122E-55A5-419C-AF66-50DC204F1BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4290" yWindow="3480" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5400" yWindow="3045" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -548,10 +548,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>软泥怪</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>送墓时：选弃牌堆1张怪物牌放在房间区任意位置或加入手牌。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -588,10 +584,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Sludge</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Metal slime</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -605,10 +597,6 @@
   </si>
   <si>
     <t>Mob slime</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Slime tower</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -701,10 +689,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>回合结束时：将本牌与同房间同侧至多1张牌一起移动1格。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>哨戒无人机</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -721,15 +705,7 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>回合结束时：如果同房间内有陷阱牌，则消灭同房间内所有陷阱牌；否则，将主牌堆或弃牌堆第1张陷阱牌加入本牌所在房间同侧，之后移动1格。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>回合结束时：选同行列其他房间对侧的1张怪物牌，使其点数减1。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>死亡时：翻开主牌堆的“史莱姆牌”直到合计点数不小于本牌点数，然后选其中1张牌加入本牌所在房间同侧，其余的牌加入手牌。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -742,11 +718,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>开战前：呼唤场上同侧所有“史莱姆”牌。&lt;br&gt;
-回合结束时：呼唤场上同侧另1张“史莱姆”牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>持续：同房间同侧所有怪物牌点数加1。&lt;br&gt;
 死亡时：本牌移动到一个同侧有怪物牌的相邻房间。</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -754,10 +725,6 @@
   <si>
     <t>回合结束时：玩家受到1伤害，然后弃置本牌。&lt;br&gt;
 开战前：呼唤弃牌堆所有同名牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>回合结束时：如果本牌所在房间没有其他牌，将本牌移动1格。否则选同房间1张其他牌，使其点数减1。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -767,11 +734,44 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>回合结束时：如果同房间同侧没有其他怪物牌，则将主牌堆第1张怪物牌加入本牌所在房间同侧，然后移动1格。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>回合结束时：将主牌堆第1张同名牌加入与本牌相邻的房间同侧。</t>
+    <t>飞溅史莱姆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>死亡时：从主牌堆翻开1张同名牌放在相邻房间同侧。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Splash slime</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>点数下降时：将主牌堆第1张“史莱姆”牌加入手牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合结束时：移动1格。然后如果同房间内有陷阱牌，则消灭同房间内1张陷阱牌；否则，从主牌堆或弃牌堆呼唤第1张陷阱牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合结束时：将本牌与同房间至多1张其他牌一起移动1格。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合结束时：移动1格。然后如果同房间有敌对怪物牌，则呼唤主牌堆第1张怪物牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Slime tower</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合结束时：呼唤主牌堆第1张同名牌到与本牌相邻的房间。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>开战前：呼唤场上所有“史莱姆”牌。&lt;br&gt;
+回合结束时：呼唤场上另1张“史莱姆”牌。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1155,22 +1155,22 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" t="s">
         <v>131</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2">
+        <v>4</v>
+      </c>
+      <c r="F2" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="C2" s="1">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2">
-        <v>4</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>133</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H2" s="3"/>
     </row>
@@ -1188,19 +1188,19 @@
         <v>4</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>7</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H3" s="3"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B4" t="s">
         <v>122</v>
@@ -1212,13 +1212,13 @@
         <v>4</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H4" s="3"/>
     </row>
@@ -1236,19 +1236,19 @@
         <v>4</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="B6" t="s">
         <v>122</v>
@@ -1260,19 +1260,19 @@
         <v>4</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H6" s="3"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B7" t="s">
         <v>122</v>
@@ -1284,10 +1284,10 @@
         <v>4</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="3"/>
@@ -1318,7 +1318,7 @@
     </row>
     <row r="9" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B9" t="s">
         <v>8</v>
@@ -1333,7 +1333,7 @@
         <v>115</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="G9" s="2" t="s">
         <v>9</v>
@@ -1378,7 +1378,7 @@
         <v>4</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="F11" s="3" t="s">
         <v>102</v>
@@ -1405,31 +1405,31 @@
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H12" s="4"/>
     </row>
-    <row r="13" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>120</v>
+        <v>169</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
       </c>
       <c r="C13" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D13" s="2">
         <v>4</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>140</v>
+        <v>171</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>16</v>
@@ -1450,7 +1450,7 @@
         <v>4</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>17</v>
@@ -1476,34 +1476,34 @@
         <v>4</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H15" s="4"/>
     </row>
-    <row r="16" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B16" t="s">
         <v>15</v>
       </c>
       <c r="C16" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D16" s="2">
         <v>4</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>135</v>
+        <v>176</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>16</v>
@@ -1512,7 +1512,7 @@
     </row>
     <row r="17" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B17" t="s">
         <v>15</v>
@@ -1524,10 +1524,10 @@
         <v>4</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>16</v>
@@ -1548,7 +1548,7 @@
         <v>4</v>
       </c>
       <c r="E18" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>4</v>
@@ -1574,7 +1574,7 @@
         <v>4</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="F19" s="3" t="s">
         <v>21</v>
@@ -1641,7 +1641,7 @@
         <v>27</v>
       </c>
       <c r="B22" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C22" s="1">
         <v>1</v>
@@ -1650,7 +1650,7 @@
         <v>4</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="F22" s="3" t="s">
         <v>29</v>
@@ -1665,16 +1665,16 @@
         <v>30</v>
       </c>
       <c r="B23" t="s">
+        <v>144</v>
+      </c>
+      <c r="C23" s="1">
+        <v>1</v>
+      </c>
+      <c r="D23" s="2">
+        <v>4</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="C23" s="1">
-        <v>1</v>
-      </c>
-      <c r="D23" s="2">
-        <v>4</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>150</v>
       </c>
       <c r="F23" s="3" t="s">
         <v>31</v>
@@ -1688,10 +1688,10 @@
     </row>
     <row r="24" spans="1:9" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B24" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C24" s="1">
         <v>2</v>
@@ -1700,7 +1700,7 @@
         <v>4</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="F24" s="3" t="s">
         <v>33</v>
@@ -1715,7 +1715,7 @@
         <v>34</v>
       </c>
       <c r="B25" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C25" s="1">
         <v>2</v>
@@ -1741,7 +1741,7 @@
         <v>0</v>
       </c>
       <c r="B26" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C26" s="1">
         <v>1</v>
@@ -1777,7 +1777,7 @@
         <v>4</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="F27" s="3" t="s">
         <v>40</v>
@@ -1803,7 +1803,7 @@
         <v>4</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="F28" s="3" t="s">
         <v>43</v>
@@ -1827,7 +1827,7 @@
         <v>4</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="F29" s="3" t="s">
         <v>47</v>
@@ -1841,10 +1841,10 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>128</v>
+      </c>
+      <c r="B30" t="s">
         <v>129</v>
-      </c>
-      <c r="B30" t="s">
-        <v>130</v>
       </c>
       <c r="C30" s="1">
         <v>1</v>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="E30" s="2"/>
       <c r="F30" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G30" s="2" t="s">
         <v>51</v>
@@ -1875,7 +1875,7 @@
         <v>4</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F31" s="3" t="s">
         <v>52</v>
@@ -1901,7 +1901,7 @@
         <v>4</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="F32" s="3" t="s">
         <v>107</v>
@@ -1925,7 +1925,7 @@
         <v>4</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>104</v>
@@ -1939,7 +1939,7 @@
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B34" t="s">
         <v>50</v>
@@ -1951,10 +1951,10 @@
         <v>4</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G34" s="2" t="s">
         <v>51</v>
@@ -1975,7 +1975,7 @@
         <v>4</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="F35" s="3" t="s">
         <v>60</v>
@@ -2001,7 +2001,7 @@
         <v>4</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>108</v>
@@ -2144,7 +2144,7 @@
         <v>4</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>80</v>

</xml_diff>

<commit_message>
Change effect of turret. Change effect of trap door.
</commit_message>
<xml_diff>
--- a/sheet/MonsterCardData.xlsx
+++ b/sheet/MonsterCardData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E6122E-55A5-419C-AF66-50DC204F1BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50840CFE-A5E1-438F-85FC-B6EC16A44D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5400" yWindow="3045" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -705,10 +705,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>回合结束时：选同行列其他房间对侧的1张怪物牌，使其点数减1。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>交锋前：弃置本牌。&lt;br&gt;
 送墓时：玩家获得3金币。</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -772,6 +768,10 @@
   <si>
     <t>开战前：呼唤场上所有“史莱姆”牌。&lt;br&gt;
 回合结束时：呼唤场上另1张“史莱姆”牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合结束时：选同行列其他房间1张敌对怪物牌，使其点数减1。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1188,7 +1188,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>7</v>
@@ -1212,7 +1212,7 @@
         <v>4</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>158</v>
@@ -1236,7 +1236,7 @@
         <v>4</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>138</v>
@@ -1260,7 +1260,7 @@
         <v>4</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>160</v>
@@ -1284,7 +1284,7 @@
         <v>4</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>162</v>
@@ -1414,7 +1414,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
@@ -1426,10 +1426,10 @@
         <v>4</v>
       </c>
       <c r="E13" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>170</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>171</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>16</v>
@@ -1450,7 +1450,7 @@
         <v>4</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>17</v>
@@ -1476,7 +1476,7 @@
         <v>4</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>133</v>
@@ -1500,10 +1500,10 @@
         <v>4</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>16</v>
@@ -1512,7 +1512,7 @@
     </row>
     <row r="17" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B17" t="s">
         <v>15</v>
@@ -1524,7 +1524,7 @@
         <v>4</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>134</v>
@@ -1925,7 +1925,7 @@
         <v>4</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F33" s="3" t="s">
         <v>104</v>
@@ -2144,7 +2144,7 @@
         <v>4</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F42" s="3" t="s">
         <v>80</v>

</xml_diff>

<commit_message>
Changed rule on turn start effect and turn end effect. Cards are flipped after using these effects and then flipped back at the end of that phase. This records which effects have already been resolved. Changed effect of bot cards. They move at turn start which gives the player some advantage.
</commit_message>
<xml_diff>
--- a/sheet/MonsterCardData.xlsx
+++ b/sheet/MonsterCardData.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50840CFE-A5E1-438F-85FC-B6EC16A44D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E200CFC-B1CD-4A42-907A-A5B10A122C28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5400" yWindow="3045" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -746,14 +746,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>回合结束时：移动1格。然后如果同房间内有陷阱牌，则消灭同房间内1张陷阱牌；否则，从主牌堆或弃牌堆呼唤第1张陷阱牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>回合结束时：将本牌与同房间至多1张其他牌一起移动1格。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>回合结束时：移动1格。然后如果同房间有敌对怪物牌，则呼唤主牌堆第1张怪物牌。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -772,6 +764,15 @@
   </si>
   <si>
     <t>回合结束时：选同行列其他房间1张敌对怪物牌，使其点数减1。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合开始时：将本牌与同房间至多1张其他牌一起移动1格。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合开始时：移动1格。&lt;br&gt;
+回合结束时：如果同房间内有陷阱牌，则消灭同房间内1张陷阱牌；否则，从主牌堆或弃牌堆呼唤第1张陷阱牌。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1174,7 +1175,7 @@
       </c>
       <c r="H2" s="3"/>
     </row>
-    <row r="3" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" ht="42.75" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
@@ -1188,7 +1189,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>7</v>
@@ -1212,7 +1213,7 @@
         <v>4</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>158</v>
@@ -1260,7 +1261,7 @@
         <v>4</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>160</v>
@@ -1284,7 +1285,7 @@
         <v>4</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>162</v>
@@ -1450,7 +1451,7 @@
         <v>4</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>17</v>
@@ -1476,7 +1477,7 @@
         <v>4</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>133</v>
@@ -1503,7 +1504,7 @@
         <v>171</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
Some bot cards' effect are not changed. Fix it.
</commit_message>
<xml_diff>
--- a/sheet/MonsterCardData.xlsx
+++ b/sheet/MonsterCardData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E200CFC-B1CD-4A42-907A-A5B10A122C28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C65E7D0-ACF2-40AB-9B10-EA425E591F56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5400" yWindow="3045" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -724,55 +724,56 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>回合结束时：移动1格。&lt;br&gt;
+    <t>飞溅史莱姆</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>死亡时：从主牌堆翻开1张同名牌放在相邻房间同侧。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Splash slime</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>点数下降时：将主牌堆第1张“史莱姆”牌加入手牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Slime tower</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合结束时：呼唤主牌堆第1张同名牌到与本牌相邻的房间。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>开战前：呼唤场上所有“史莱姆”牌。&lt;br&gt;
+回合结束时：呼唤场上另1张“史莱姆”牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合结束时：选同行列其他房间1张敌对怪物牌，使其点数减1。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合开始时：将本牌与同房间至多1张其他牌一起移动1格。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合开始时：移动1格。&lt;br&gt;
+回合结束时：如果同房间内有陷阱牌，则消灭同房间内1张陷阱牌；否则，从主牌堆或弃牌堆呼唤第1张陷阱牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>回合开始时：移动1格。&lt;br&gt;
 移动时：点数减1。&lt;br&gt;
 点数为0而被消灭时：使同房间内所有其他牌点数减1，然后玩家受到1伤害。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>飞溅史莱姆</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>死亡时：从主牌堆翻开1张同名牌放在相邻房间同侧。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Splash slime</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>点数下降时：将主牌堆第1张“史莱姆”牌加入手牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>回合结束时：移动1格。然后如果同房间有敌对怪物牌，则呼唤主牌堆第1张怪物牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Slime tower</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>回合结束时：呼唤主牌堆第1张同名牌到与本牌相邻的房间。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>开战前：呼唤场上所有“史莱姆”牌。&lt;br&gt;
-回合结束时：呼唤场上另1张“史莱姆”牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>回合结束时：选同行列其他房间1张敌对怪物牌，使其点数减1。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>回合开始时：将本牌与同房间至多1张其他牌一起移动1格。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>回合开始时：移动1格。&lt;br&gt;
-回合结束时：如果同房间内有陷阱牌，则消灭同房间内1张陷阱牌；否则，从主牌堆或弃牌堆呼唤第1张陷阱牌。</t>
+回合结束时：如果同房间有敌对怪物牌，则呼唤主牌堆第1张怪物牌。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1189,7 +1190,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>7</v>
@@ -1213,7 +1214,7 @@
         <v>4</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F4" s="3" t="s">
         <v>158</v>
@@ -1231,13 +1232,13 @@
         <v>122</v>
       </c>
       <c r="C5" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="2">
         <v>4</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="F5" s="3" t="s">
         <v>138</v>
@@ -1247,7 +1248,7 @@
       </c>
       <c r="H5" s="3"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>159</v>
       </c>
@@ -1261,7 +1262,7 @@
         <v>4</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>160</v>
@@ -1285,7 +1286,7 @@
         <v>4</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>162</v>
@@ -1415,7 +1416,7 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B13" t="s">
         <v>15</v>
@@ -1427,10 +1428,10 @@
         <v>4</v>
       </c>
       <c r="E13" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>169</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>170</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>16</v>
@@ -1451,7 +1452,7 @@
         <v>4</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>17</v>
@@ -1477,7 +1478,7 @@
         <v>4</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>133</v>
@@ -1501,10 +1502,10 @@
         <v>4</v>
       </c>
       <c r="E16" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>171</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>173</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>16</v>

</xml_diff>

<commit_message>
Fixed some rank-changing continuous effect: They get ambiguous when combined with move effect and effect concerned about rank, such as Kamikaze Bot. Modified these effects to clarify them. Quicksand is changed to -> On engage start: Change rank of all cards in its territory to 1. Swamp is changed to -> On turn end: Reduce the rank of all cards in its territory by 1 whose rank is higher than 1. Card effect change: Splash Slime -> Can only rally in adjacent room where at least an ally exists now. Duel -> now set its rank to the rank of the avatar card it replaced. Card change: Lowered the rank of some skill cards. Rule change: Clarify that territory cards' on turn start/end effect resolves before those in the floor zone.
</commit_message>
<xml_diff>
--- a/sheet/MonsterCardData.xlsx
+++ b/sheet/MonsterCardData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\nanDeck\DungeonCrawlDeckMaster\sheet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03C42B0A-A623-4410-A0CA-846D9880640C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFA8FCF8-7E4D-4645-8AFE-3110695F51BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -745,11 +745,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>持续：同房间所有友方怪物牌点数加1。&lt;br&gt;
-死亡时：移动到一个有友方怪物牌的相邻房间并免死。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>枪手</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -788,16 +783,21 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
+    <t>回合结束时：召集主牌堆第1张同名牌到与本牌相邻的房间。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>开战前：召集所有相邻房间的所有“史莱姆”牌。&lt;br&gt;
-回合结束时：召集相邻房间的1张“史莱姆”牌。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>回合结束时：召集主牌堆第1张同名牌到与本牌相邻的房间。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>死亡时：召集1张同名牌到相邻房间。</t>
+回合结束时：召集1个相邻房间的1张“史莱姆”牌。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>持续：同房间所有友方怪物牌点数加1。&lt;br&gt;
+死亡时：移动到1个有友方怪物牌的相邻房间并免死。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>死亡时：召集1张同名牌到1个相邻房间，该房间必须有友方的牌。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1214,7 +1214,7 @@
         <v>4</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>7</v>
@@ -1286,7 +1286,7 @@
         <v>4</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>160</v>
@@ -1310,7 +1310,7 @@
         <v>4</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>162</v>
@@ -1502,7 +1502,7 @@
         <v>4</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>133</v>
@@ -1614,7 +1614,7 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B20" t="s">
         <v>20</v>
@@ -1626,7 +1626,7 @@
         <v>4</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="2"/>
@@ -1634,7 +1634,7 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B21" t="s">
         <v>92</v>
@@ -1646,7 +1646,7 @@
         <v>4</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F21" s="3"/>
       <c r="G21" s="2"/>
@@ -1654,7 +1654,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B22" t="s">
         <v>20</v>
@@ -1666,7 +1666,7 @@
         <v>4</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F22" s="3"/>
       <c r="G22" s="2"/>
@@ -2011,7 +2011,7 @@
         <v>4</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="F36" s="3" t="s">
         <v>104</v>

</xml_diff>